<commit_message>
added format cleanup script to test
</commit_message>
<xml_diff>
--- a/test-files/2000-preformatted-errs.xlsx
+++ b/test-files/2000-preformatted-errs.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stateofdelaware-my.sharepoint.com/personal/bryan_snyder_delaware_gov/Documents/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\leading-zeros-dates\test-files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="11_2BB1D69C5B0058CCCC21D693523088B35299F59A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{63DF516F-A419-48CC-8E5C-6A1A26E16161}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B270DE8B-A274-462E-975A-B72357512676}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2670" yWindow="3270" windowWidth="38700" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10710" yWindow="2805" windowWidth="38700" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,10 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="20">
-  <si>
-    <t>FullDate</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="21">
   <si>
     <t>04/14/2004 - 05/31/2008</t>
   </si>
@@ -61,25 +58,31 @@
     <t>01/02/1999 - 03/15/2002</t>
   </si>
   <si>
+    <t>01/01/1999 - 03/31/2002</t>
+  </si>
+  <si>
     <t>4/14/2010 - 5/31/2008</t>
   </si>
   <si>
     <t>4/14/2004 - 5/31/2008</t>
   </si>
   <si>
+    <t>04/14/2004 - 04/30/2008</t>
+  </si>
+  <si>
     <t>6/1/2008 - 10/30/2009</t>
   </si>
   <si>
-    <t>ExpectedResult</t>
-  </si>
-  <si>
-    <t>ErrorOutputs</t>
-  </si>
-  <si>
-    <t>04/14/2004 - 04/30/2008</t>
-  </si>
-  <si>
     <t>06/01/2008 - 10/31/2009</t>
+  </si>
+  <si>
+    <t>Input</t>
+  </si>
+  <si>
+    <t>ExpectedOutput</t>
+  </si>
+  <si>
+    <t>ActualOutput</t>
   </si>
 </sst>
 </file>
@@ -100,18 +103,12 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -141,12 +138,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -162,10 +158,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -456,115 +448,116 @@
   <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.42578125" customWidth="1"/>
-    <col min="3" max="3" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="3" width="22.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="B2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="2" t="s">
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+      <c r="B3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" t="s">
         <v>3</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>8</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B8" t="s">
         <v>8</v>
       </c>
-      <c r="C7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
+      <c r="C8" t="s">
         <v>9</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B10" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" t="s">
         <v>12</v>
       </c>
     </row>
@@ -573,6 +566,9 @@
         <v>13</v>
       </c>
       <c r="B11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C11" t="s">
         <v>9</v>
       </c>
     </row>
@@ -581,15 +577,21 @@
         <v>14</v>
       </c>
       <c r="B12" t="s">
-        <v>18</v>
+        <v>15</v>
+      </c>
+      <c r="C12" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B13" t="s">
-        <v>19</v>
+        <v>17</v>
+      </c>
+      <c r="C13" t="s">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated to handle serial dates
</commit_message>
<xml_diff>
--- a/test-files/2000-preformatted-errs.xlsx
+++ b/test-files/2000-preformatted-errs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\leading-zeros-dates\test-files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B270DE8B-A274-462E-975A-B72357512676}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{020CA3A5-9758-49FE-B5E5-0D51065C8822}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10710" yWindow="2805" windowWidth="38700" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5805" yWindow="3090" windowWidth="18180" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,28 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="27">
+  <si>
+    <t>Correct</t>
+  </si>
+  <si>
+    <t>Input</t>
+  </si>
+  <si>
+    <t>ExpectedOutput</t>
+  </si>
+  <si>
+    <t>LastError</t>
+  </si>
+  <si>
+    <t>FormattedInput</t>
+  </si>
+  <si>
+    <t>Check Me</t>
+  </si>
+  <si>
+    <t>y</t>
+  </si>
   <si>
     <t>04/14/2004 - 05/31/2008</t>
   </si>
@@ -52,6 +73,9 @@
     <t>05/30/2008 - 04/01/2010</t>
   </si>
   <si>
+    <t>05/31/2008 - 04/14/2010</t>
+  </si>
+  <si>
     <t>04/14/1998 - 05/31/1999</t>
   </si>
   <si>
@@ -61,6 +85,9 @@
     <t>01/01/1999 - 03/31/2002</t>
   </si>
   <si>
+    <t>n</t>
+  </si>
+  <si>
     <t>4/14/2010 - 5/31/2008</t>
   </si>
   <si>
@@ -74,15 +101,6 @@
   </si>
   <si>
     <t>06/01/2008 - 10/31/2009</t>
-  </si>
-  <si>
-    <t>Input</t>
-  </si>
-  <si>
-    <t>ExpectedOutput</t>
-  </si>
-  <si>
-    <t>ActualOutput</t>
   </si>
 </sst>
 </file>
@@ -445,153 +463,236 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="3" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="5" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D9" t="s">
+        <v>18</v>
+      </c>
+      <c r="E9" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" t="s">
         <v>19</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C10" t="s">
+        <v>19</v>
+      </c>
+      <c r="D10" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
-        <v>2</v>
-      </c>
-      <c r="C3" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="E10" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11" t="s">
+        <v>15</v>
+      </c>
+      <c r="D11" t="s">
+        <v>16</v>
+      </c>
+      <c r="E11" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" t="s">
+        <v>24</v>
+      </c>
+      <c r="D12" t="s">
+        <v>8</v>
+      </c>
+      <c r="E12" t="s">
         <v>7</v>
       </c>
-      <c r="B7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C7" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" t="s">
+        <v>25</v>
+      </c>
+      <c r="C13" t="s">
+        <v>26</v>
+      </c>
+      <c r="D13" t="s">
         <v>10</v>
       </c>
-      <c r="B9" t="s">
+      <c r="E13" t="s">
         <v>10</v>
-      </c>
-      <c r="C9" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>11</v>
-      </c>
-      <c r="B10" t="s">
-        <v>11</v>
-      </c>
-      <c r="C10" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>13</v>
-      </c>
-      <c r="B11" t="s">
-        <v>8</v>
-      </c>
-      <c r="C11" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>14</v>
-      </c>
-      <c r="B12" t="s">
-        <v>15</v>
-      </c>
-      <c r="C12" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>16</v>
-      </c>
-      <c r="B13" t="s">
-        <v>17</v>
-      </c>
-      <c r="C13" t="s">
-        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>